<commit_message>
DB: CropTable.csv 수정, CropSeasonMulTable.csv 추가, EggEffectTable.csv 프로토타입 추가(정식 사용 x)
</commit_message>
<xml_diff>
--- a/Assets/Project/Csv/Crop/CropTable.xlsx
+++ b/Assets/Project/Csv/Crop/CropTable.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ycjun\OneDrive\문서\Projects\Git\Dairy Farm\Assets\Project\Csv\Crop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C8F967-ED5E-4275-A19D-77A75A84DC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF475BD-23BF-423A-803C-DF0A2C420526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="DataTabel" sheetId="1" r:id="rId1"/>
+    <sheet name="enum Season" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>{id/int/UNIQUE/NOT NULL}</t>
   </si>
@@ -37,52 +38,67 @@
     <t>{growthSpriteIds/AssetID[]/NOT NULL}</t>
   </si>
   <si>
+    <t>{seedId/int/UNIQUE/NOT NULL}</t>
+  </si>
+  <si>
     <t>{seedName/string/UNIQUE/NOT NULL}</t>
   </si>
   <si>
+    <t>벼</t>
+  </si>
+  <si>
+    <t>1|2</t>
+  </si>
+  <si>
+    <t>볍씨</t>
+  </si>
+  <si>
     <t>토마토</t>
   </si>
   <si>
+    <t>2|4</t>
+  </si>
+  <si>
+    <t>토마토 씨앗</t>
+  </si>
+  <si>
     <t>호박</t>
   </si>
   <si>
+    <t>3|6</t>
+  </si>
+  <si>
+    <t>호박 씨앗</t>
+  </si>
+  <si>
     <t>딸기</t>
   </si>
   <si>
-    <t>{seedId/int/UNIQUE/NOT NULL}</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>쌀</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>볍씨</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>토마토 씨앗</t>
-  </si>
-  <si>
-    <t>호박 씨앗</t>
+    <t>4|7</t>
   </si>
   <si>
     <t>딸기 씨앗</t>
   </si>
   <si>
-    <t>1|2</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2|4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>3|6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>4|7</t>
+    <t>enum Season</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t>Summer</t>
+  </si>
+  <si>
+    <t>Autumn</t>
+  </si>
+  <si>
+    <t>Winter</t>
+  </si>
+  <si>
+    <t>{defaultYieldCount/int/NOT NULL}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -180,7 +196,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -206,6 +222,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -540,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.625" style="1" bestFit="1" customWidth="1"/>
@@ -548,11 +565,12 @@
     <col min="3" max="3" width="25.375" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.5" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="36.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="31.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.25" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.125" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -569,18 +587,21 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="8">
         <v>1000</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
@@ -589,21 +610,24 @@
         <v>7</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F2" s="6">
         <v>100</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+      <c r="H2" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1100</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3">
         <v>1</v>
@@ -612,7 +636,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F3" s="6">
         <v>110</v>
@@ -620,13 +644,16 @@
       <c r="G3" s="6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1200</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3">
         <v>2</v>
@@ -635,21 +662,24 @@
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F4" s="6">
         <v>120</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1300</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3">
         <v>3</v>
@@ -658,13 +688,71 @@
         <v>1</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="6">
         <v>130</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>14</v>
+        <v>18</v>
+      </c>
+      <c r="H5" s="3">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" style="1" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>